<commit_message>
HFA task types pre-filled; leave on a firm holiday no longer counted twice
- The template's Task Types tab now ships with HFA's 46 Karbon task types
  (src/roster/hfa-task-types.ts): billability as Karbon marks it; Bereavement,
  Jury Duty, PTO - Holiday and PTO - Vacation as PTO; PTO - Sick as Sick.
  Checked one-for-one against the owner's list.
- Minimal-entry line: PTO logged on a firm holiday (a "PTO - Holiday" code)
  lowered the line a second time on top of the Holidays tab — a full-timer's
  holiday-week line fell from 16 h to 12 h. Leave on a firm holiday now
  doesn't count again. Regression test added.
- Decision 26 (incl. two types to confirm: Admin and "Preparation & Review
  of your Individual Income Tax Return" are billable in Karbon); go-live and
  README updated; template rebuilt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JQUVYxXwNTEL9NcvWSp8Gk
</commit_message>
<xml_diff>
--- a/templates/HFA_Staff_Roster_Template.xlsx
+++ b/templates/HFA_Staff_Roster_Template.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="97">
   <si>
     <t>Blue rows are examples — replace with real data. Department, Status, CSA Assigned and Exclude use dropdowns (see Lists). Target is a percent (80). Blank Expected Weekly Hours = full time.</t>
   </si>
@@ -119,7 +119,7 @@
     <t>Karbon Client ID</t>
   </si>
   <si>
-    <t>Every Karbon task type, with how it counts. Run `pnpm tg karbon:task-types` to list the task types used in Karbon recently; any type missing here is reported each week.</t>
+    <t>HFA’s Karbon task types, pre-filled (billability as Karbon sets it). Run `pnpm tg karbon:task-types` to check them against Karbon; a new or renamed type missing here is reported each week.</t>
   </si>
   <si>
     <t>Task Type</t>
@@ -128,6 +128,153 @@
     <t>Category</t>
   </si>
   <si>
+    <t>Admin</t>
+  </si>
+  <si>
+    <t>Billable</t>
+  </si>
+  <si>
+    <t>Administrative</t>
+  </si>
+  <si>
+    <t>Non-billable</t>
+  </si>
+  <si>
+    <t>Advisory Services</t>
+  </si>
+  <si>
+    <t>AUP Procedures</t>
+  </si>
+  <si>
+    <t>Bereavement</t>
+  </si>
+  <si>
+    <t>PTO</t>
+  </si>
+  <si>
+    <t>Business Advisory</t>
+  </si>
+  <si>
+    <t>Business Development/Marketing</t>
+  </si>
+  <si>
+    <t>CAS - Accounting / Bookkeeping</t>
+  </si>
+  <si>
+    <t>CAS - BPO - Back Office Process Outsourcing</t>
+  </si>
+  <si>
+    <t>CAS - CFO Services</t>
+  </si>
+  <si>
+    <t>CAS - Controllership Services</t>
+  </si>
+  <si>
+    <t>CAS - Financial Planning &amp; Analysis</t>
+  </si>
+  <si>
+    <t>Client / Project Setup</t>
+  </si>
+  <si>
+    <t>Client Meeting / Communication</t>
+  </si>
+  <si>
+    <t>Client Training</t>
+  </si>
+  <si>
+    <t>Committees - Fun Club</t>
+  </si>
+  <si>
+    <t>Committees - Practice Dev</t>
+  </si>
+  <si>
+    <t>Committees - Quality Control</t>
+  </si>
+  <si>
+    <t>Committees - Technology</t>
+  </si>
+  <si>
+    <t>Committees - Training &amp; Dev</t>
+  </si>
+  <si>
+    <t>Community Impact</t>
+  </si>
+  <si>
+    <t>Compliance</t>
+  </si>
+  <si>
+    <t>Down!</t>
+  </si>
+  <si>
+    <t>Employee Engagement</t>
+  </si>
+  <si>
+    <t>Fieldwork</t>
+  </si>
+  <si>
+    <t>Financial Operations (Internal)</t>
+  </si>
+  <si>
+    <t>Internal Meetings</t>
+  </si>
+  <si>
+    <t>Jury Duty</t>
+  </si>
+  <si>
+    <t>Non-Attest Work</t>
+  </si>
+  <si>
+    <t>Personnel Development</t>
+  </si>
+  <si>
+    <t>Planning</t>
+  </si>
+  <si>
+    <t>Practice Development</t>
+  </si>
+  <si>
+    <t>Preparation &amp; Review of your Individual Income Tax Return</t>
+  </si>
+  <si>
+    <t>Processing</t>
+  </si>
+  <si>
+    <t>Professional Development &amp; Training</t>
+  </si>
+  <si>
+    <t>PTO - Holiday</t>
+  </si>
+  <si>
+    <t>PTO - Sick</t>
+  </si>
+  <si>
+    <t>Sick</t>
+  </si>
+  <si>
+    <t>PTO - Vacation</t>
+  </si>
+  <si>
+    <t>Report Preparation</t>
+  </si>
+  <si>
+    <t>Research - Billable</t>
+  </si>
+  <si>
+    <t>Review</t>
+  </si>
+  <si>
+    <t>Tax Preparation</t>
+  </si>
+  <si>
+    <t>Tax Review</t>
+  </si>
+  <si>
+    <t>Training</t>
+  </si>
+  <si>
+    <t>Travel</t>
+  </si>
+  <si>
     <t>Firm holidays. A weekday holiday lowers that week’s minimal-time line and the month’s capacity.</t>
   </si>
   <si>
@@ -143,9 +290,6 @@
     <t>Yes/No</t>
   </si>
   <si>
-    <t>Billable</t>
-  </si>
-  <si>
     <t>Yes</t>
   </si>
   <si>
@@ -155,25 +299,13 @@
     <t>Inactive</t>
   </si>
   <si>
-    <t>Non-billable</t>
-  </si>
-  <si>
     <t>Partner</t>
   </si>
   <si>
     <t>CSA-3</t>
   </si>
   <si>
-    <t>PTO</t>
-  </si>
-  <si>
     <t>Advisory</t>
-  </si>
-  <si>
-    <t>Sick</t>
-  </si>
-  <si>
-    <t>Admin</t>
   </si>
 </sst>
 </file>
@@ -2835,7 +2967,7 @@
   <dimension ref="A1:B500"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="40" customWidth="1"/>
+    <col min="1" max="1" width="52" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2853,52 +2985,374 @@
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="5" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="7" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="8" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="9" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="10" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="11" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="15" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="22" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="23" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="24" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="25" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="29" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="30" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="31" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="32" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="33" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="34" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="35" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="36" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="37" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="38" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="39" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="40" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="41" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="42" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="43" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="44" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="45" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="46" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="47" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="48" spans="2:2" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B9" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>46</v>
+      </c>
+      <c r="B10" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>47</v>
+      </c>
+      <c r="B11" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>48</v>
+      </c>
+      <c r="B12" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>49</v>
+      </c>
+      <c r="B13" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>50</v>
+      </c>
+      <c r="B14" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>51</v>
+      </c>
+      <c r="B15" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>52</v>
+      </c>
+      <c r="B16" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>53</v>
+      </c>
+      <c r="B17" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>54</v>
+      </c>
+      <c r="B18" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>55</v>
+      </c>
+      <c r="B19" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>56</v>
+      </c>
+      <c r="B20" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>57</v>
+      </c>
+      <c r="B21" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>58</v>
+      </c>
+      <c r="B22" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>59</v>
+      </c>
+      <c r="B23" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>60</v>
+      </c>
+      <c r="B24" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>61</v>
+      </c>
+      <c r="B25" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>62</v>
+      </c>
+      <c r="B26" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>63</v>
+      </c>
+      <c r="B27" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>64</v>
+      </c>
+      <c r="B28" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>65</v>
+      </c>
+      <c r="B29" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>66</v>
+      </c>
+      <c r="B30" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>67</v>
+      </c>
+      <c r="B31" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>68</v>
+      </c>
+      <c r="B32" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>69</v>
+      </c>
+      <c r="B33" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>70</v>
+      </c>
+      <c r="B34" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>71</v>
+      </c>
+      <c r="B35" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>72</v>
+      </c>
+      <c r="B36" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B37" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>74</v>
+      </c>
+      <c r="B38" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>75</v>
+      </c>
+      <c r="B39" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>76</v>
+      </c>
+      <c r="B40" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>78</v>
+      </c>
+      <c r="B41" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>79</v>
+      </c>
+      <c r="B42" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>80</v>
+      </c>
+      <c r="B43" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>81</v>
+      </c>
+      <c r="B44" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>82</v>
+      </c>
+      <c r="B45" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>83</v>
+      </c>
+      <c r="B46" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>84</v>
+      </c>
+      <c r="B47" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>85</v>
+      </c>
+      <c r="B48" t="s">
+        <v>40</v>
+      </c>
+    </row>
     <row r="49" spans="2:2" x14ac:dyDescent="0.25"/>
     <row r="50" spans="2:2" x14ac:dyDescent="0.25"/>
     <row r="51" spans="2:2" x14ac:dyDescent="0.25"/>
@@ -3379,16 +3833,16 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>37</v>
+        <v>86</v>
       </c>
       <c r="B1" s="1"/>
     </row>
     <row r="2" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>38</v>
+        <v>87</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>39</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
@@ -3707,7 +4161,7 @@
   <sheetData>
     <row r="1" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>40</v>
+        <v>89</v>
       </c>
       <c r="B1" s="7" t="s">
         <v>6</v>
@@ -3719,7 +4173,7 @@
         <v>36</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>41</v>
+        <v>90</v>
       </c>
       <c r="F1" s="7" t="s">
         <v>30</v>
@@ -3736,13 +4190,13 @@
         <v>16</v>
       </c>
       <c r="D2" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="E2" t="s">
-        <v>43</v>
+        <v>91</v>
       </c>
       <c r="F2" t="s">
-        <v>44</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -3750,19 +4204,19 @@
         <v>22</v>
       </c>
       <c r="B3" t="s">
-        <v>45</v>
+        <v>93</v>
       </c>
       <c r="C3" t="s">
         <v>27</v>
       </c>
       <c r="D3" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="E3" t="s">
         <v>19</v>
       </c>
       <c r="F3" t="s">
-        <v>47</v>
+        <v>94</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -3770,10 +4224,10 @@
         <v>25</v>
       </c>
       <c r="C4" t="s">
-        <v>48</v>
+        <v>95</v>
       </c>
       <c r="D4" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="F4" t="s">
         <v>4</v>
@@ -3781,15 +4235,15 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>50</v>
+        <v>96</v>
       </c>
       <c r="D5" t="s">
-        <v>51</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Task types: drop Admin and own-return prep (being deleted from Karbon); 44 types
Bereavement and Jury Duty confirmed as PTO. Decision 26 and go-live updated;
template rebuilt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JQUVYxXwNTEL9NcvWSp8Gk
</commit_message>
<xml_diff>
--- a/templates/HFA_Staff_Roster_Template.xlsx
+++ b/templates/HFA_Staff_Roster_Template.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="96">
   <si>
     <t>Blue rows are examples — replace with real data. Department, Status, CSA Assigned and Exclude use dropdowns (see Lists). Target is a percent (80). Blank Expected Weekly Hours = full time.</t>
   </si>
@@ -128,184 +128,181 @@
     <t>Category</t>
   </si>
   <si>
+    <t>Administrative</t>
+  </si>
+  <si>
+    <t>Non-billable</t>
+  </si>
+  <si>
+    <t>Advisory Services</t>
+  </si>
+  <si>
+    <t>Billable</t>
+  </si>
+  <si>
+    <t>AUP Procedures</t>
+  </si>
+  <si>
+    <t>Bereavement</t>
+  </si>
+  <si>
+    <t>PTO</t>
+  </si>
+  <si>
+    <t>Business Advisory</t>
+  </si>
+  <si>
+    <t>Business Development/Marketing</t>
+  </si>
+  <si>
+    <t>CAS - Accounting / Bookkeeping</t>
+  </si>
+  <si>
+    <t>CAS - BPO - Back Office Process Outsourcing</t>
+  </si>
+  <si>
+    <t>CAS - CFO Services</t>
+  </si>
+  <si>
+    <t>CAS - Controllership Services</t>
+  </si>
+  <si>
+    <t>CAS - Financial Planning &amp; Analysis</t>
+  </si>
+  <si>
+    <t>Client / Project Setup</t>
+  </si>
+  <si>
+    <t>Client Meeting / Communication</t>
+  </si>
+  <si>
+    <t>Client Training</t>
+  </si>
+  <si>
+    <t>Committees - Fun Club</t>
+  </si>
+  <si>
+    <t>Committees - Practice Dev</t>
+  </si>
+  <si>
+    <t>Committees - Quality Control</t>
+  </si>
+  <si>
+    <t>Committees - Technology</t>
+  </si>
+  <si>
+    <t>Committees - Training &amp; Dev</t>
+  </si>
+  <si>
+    <t>Community Impact</t>
+  </si>
+  <si>
+    <t>Compliance</t>
+  </si>
+  <si>
+    <t>Down!</t>
+  </si>
+  <si>
+    <t>Employee Engagement</t>
+  </si>
+  <si>
+    <t>Fieldwork</t>
+  </si>
+  <si>
+    <t>Financial Operations (Internal)</t>
+  </si>
+  <si>
+    <t>Internal Meetings</t>
+  </si>
+  <si>
+    <t>Jury Duty</t>
+  </si>
+  <si>
+    <t>Non-Attest Work</t>
+  </si>
+  <si>
+    <t>Personnel Development</t>
+  </si>
+  <si>
+    <t>Planning</t>
+  </si>
+  <si>
+    <t>Practice Development</t>
+  </si>
+  <si>
+    <t>Processing</t>
+  </si>
+  <si>
+    <t>Professional Development &amp; Training</t>
+  </si>
+  <si>
+    <t>PTO - Holiday</t>
+  </si>
+  <si>
+    <t>PTO - Sick</t>
+  </si>
+  <si>
+    <t>Sick</t>
+  </si>
+  <si>
+    <t>PTO - Vacation</t>
+  </si>
+  <si>
+    <t>Report Preparation</t>
+  </si>
+  <si>
+    <t>Research - Billable</t>
+  </si>
+  <si>
+    <t>Review</t>
+  </si>
+  <si>
+    <t>Tax Preparation</t>
+  </si>
+  <si>
+    <t>Tax Review</t>
+  </si>
+  <si>
+    <t>Training</t>
+  </si>
+  <si>
+    <t>Travel</t>
+  </si>
+  <si>
+    <t>Firm holidays. A weekday holiday lowers that week’s minimal-time line and the month’s capacity.</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Holiday</t>
+  </si>
+  <si>
+    <t>Departments</t>
+  </si>
+  <si>
+    <t>Yes/No</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>CSA</t>
+  </si>
+  <si>
+    <t>Inactive</t>
+  </si>
+  <si>
+    <t>Partner</t>
+  </si>
+  <si>
+    <t>CSA-3</t>
+  </si>
+  <si>
+    <t>Advisory</t>
+  </si>
+  <si>
     <t>Admin</t>
-  </si>
-  <si>
-    <t>Billable</t>
-  </si>
-  <si>
-    <t>Administrative</t>
-  </si>
-  <si>
-    <t>Non-billable</t>
-  </si>
-  <si>
-    <t>Advisory Services</t>
-  </si>
-  <si>
-    <t>AUP Procedures</t>
-  </si>
-  <si>
-    <t>Bereavement</t>
-  </si>
-  <si>
-    <t>PTO</t>
-  </si>
-  <si>
-    <t>Business Advisory</t>
-  </si>
-  <si>
-    <t>Business Development/Marketing</t>
-  </si>
-  <si>
-    <t>CAS - Accounting / Bookkeeping</t>
-  </si>
-  <si>
-    <t>CAS - BPO - Back Office Process Outsourcing</t>
-  </si>
-  <si>
-    <t>CAS - CFO Services</t>
-  </si>
-  <si>
-    <t>CAS - Controllership Services</t>
-  </si>
-  <si>
-    <t>CAS - Financial Planning &amp; Analysis</t>
-  </si>
-  <si>
-    <t>Client / Project Setup</t>
-  </si>
-  <si>
-    <t>Client Meeting / Communication</t>
-  </si>
-  <si>
-    <t>Client Training</t>
-  </si>
-  <si>
-    <t>Committees - Fun Club</t>
-  </si>
-  <si>
-    <t>Committees - Practice Dev</t>
-  </si>
-  <si>
-    <t>Committees - Quality Control</t>
-  </si>
-  <si>
-    <t>Committees - Technology</t>
-  </si>
-  <si>
-    <t>Committees - Training &amp; Dev</t>
-  </si>
-  <si>
-    <t>Community Impact</t>
-  </si>
-  <si>
-    <t>Compliance</t>
-  </si>
-  <si>
-    <t>Down!</t>
-  </si>
-  <si>
-    <t>Employee Engagement</t>
-  </si>
-  <si>
-    <t>Fieldwork</t>
-  </si>
-  <si>
-    <t>Financial Operations (Internal)</t>
-  </si>
-  <si>
-    <t>Internal Meetings</t>
-  </si>
-  <si>
-    <t>Jury Duty</t>
-  </si>
-  <si>
-    <t>Non-Attest Work</t>
-  </si>
-  <si>
-    <t>Personnel Development</t>
-  </si>
-  <si>
-    <t>Planning</t>
-  </si>
-  <si>
-    <t>Practice Development</t>
-  </si>
-  <si>
-    <t>Preparation &amp; Review of your Individual Income Tax Return</t>
-  </si>
-  <si>
-    <t>Processing</t>
-  </si>
-  <si>
-    <t>Professional Development &amp; Training</t>
-  </si>
-  <si>
-    <t>PTO - Holiday</t>
-  </si>
-  <si>
-    <t>PTO - Sick</t>
-  </si>
-  <si>
-    <t>Sick</t>
-  </si>
-  <si>
-    <t>PTO - Vacation</t>
-  </si>
-  <si>
-    <t>Report Preparation</t>
-  </si>
-  <si>
-    <t>Research - Billable</t>
-  </si>
-  <si>
-    <t>Review</t>
-  </si>
-  <si>
-    <t>Tax Preparation</t>
-  </si>
-  <si>
-    <t>Tax Review</t>
-  </si>
-  <si>
-    <t>Training</t>
-  </si>
-  <si>
-    <t>Travel</t>
-  </si>
-  <si>
-    <t>Firm holidays. A weekday holiday lowers that week’s minimal-time line and the month’s capacity.</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>Holiday</t>
-  </si>
-  <si>
-    <t>Departments</t>
-  </si>
-  <si>
-    <t>Yes/No</t>
-  </si>
-  <si>
-    <t>Yes</t>
-  </si>
-  <si>
-    <t>CSA</t>
-  </si>
-  <si>
-    <t>Inactive</t>
-  </si>
-  <si>
-    <t>Partner</t>
-  </si>
-  <si>
-    <t>CSA-3</t>
-  </si>
-  <si>
-    <t>Advisory</t>
   </si>
 </sst>
 </file>
@@ -3006,7 +3003,7 @@
         <v>41</v>
       </c>
       <c r="B5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -3014,23 +3011,23 @@
         <v>42</v>
       </c>
       <c r="B6" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>43</v>
+        <v>25</v>
       </c>
       <c r="B7" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>25</v>
+        <v>44</v>
       </c>
       <c r="B8" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -3054,7 +3051,7 @@
         <v>47</v>
       </c>
       <c r="B11" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -3062,7 +3059,7 @@
         <v>48</v>
       </c>
       <c r="B12" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -3070,7 +3067,7 @@
         <v>49</v>
       </c>
       <c r="B13" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -3078,7 +3075,7 @@
         <v>50</v>
       </c>
       <c r="B14" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -3086,7 +3083,7 @@
         <v>51</v>
       </c>
       <c r="B15" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -3094,7 +3091,7 @@
         <v>52</v>
       </c>
       <c r="B16" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -3102,7 +3099,7 @@
         <v>53</v>
       </c>
       <c r="B17" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -3118,7 +3115,7 @@
         <v>55</v>
       </c>
       <c r="B19" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -3126,7 +3123,7 @@
         <v>56</v>
       </c>
       <c r="B20" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -3134,7 +3131,7 @@
         <v>57</v>
       </c>
       <c r="B21" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -3142,7 +3139,7 @@
         <v>58</v>
       </c>
       <c r="B22" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -3150,7 +3147,7 @@
         <v>59</v>
       </c>
       <c r="B23" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
@@ -3174,7 +3171,7 @@
         <v>62</v>
       </c>
       <c r="B26" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
@@ -3198,7 +3195,7 @@
         <v>65</v>
       </c>
       <c r="B29" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
@@ -3206,7 +3203,7 @@
         <v>66</v>
       </c>
       <c r="B30" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
@@ -3214,7 +3211,7 @@
         <v>67</v>
       </c>
       <c r="B31" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
@@ -3262,7 +3259,7 @@
         <v>73</v>
       </c>
       <c r="B37" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
@@ -3270,23 +3267,23 @@
         <v>74</v>
       </c>
       <c r="B38" t="s">
-        <v>40</v>
+        <v>75</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B39" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B40" t="s">
-        <v>77</v>
+        <v>40</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
@@ -3294,7 +3291,7 @@
         <v>78</v>
       </c>
       <c r="B41" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
@@ -3302,7 +3299,7 @@
         <v>79</v>
       </c>
       <c r="B42" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
@@ -3310,7 +3307,7 @@
         <v>80</v>
       </c>
       <c r="B43" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
@@ -3318,7 +3315,7 @@
         <v>81</v>
       </c>
       <c r="B44" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
@@ -3337,22 +3334,8 @@
         <v>38</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>84</v>
-      </c>
-      <c r="B47" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>85</v>
-      </c>
-      <c r="B48" t="s">
-        <v>40</v>
-      </c>
-    </row>
+    <row r="47" spans="2:2" x14ac:dyDescent="0.25"/>
+    <row r="48" spans="2:2" x14ac:dyDescent="0.25"/>
     <row r="49" spans="2:2" x14ac:dyDescent="0.25"/>
     <row r="50" spans="2:2" x14ac:dyDescent="0.25"/>
     <row r="51" spans="2:2" x14ac:dyDescent="0.25"/>
@@ -3833,16 +3816,16 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B1" s="1"/>
     </row>
     <row r="2" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
@@ -4161,7 +4144,7 @@
   <sheetData>
     <row r="1" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B1" s="7" t="s">
         <v>6</v>
@@ -4173,7 +4156,7 @@
         <v>36</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="F1" s="7" t="s">
         <v>30</v>
@@ -4190,13 +4173,13 @@
         <v>16</v>
       </c>
       <c r="D2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="F2" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -4204,19 +4187,19 @@
         <v>22</v>
       </c>
       <c r="B3" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C3" t="s">
         <v>27</v>
       </c>
       <c r="D3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E3" t="s">
         <v>19</v>
       </c>
       <c r="F3" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -4224,10 +4207,10 @@
         <v>25</v>
       </c>
       <c r="C4" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F4" t="s">
         <v>4</v>
@@ -4235,15 +4218,15 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D5" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>37</v>
+        <v>95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>